<commit_message>
test(smt-layout): cover isolated BOM uploads
</commit_message>
<xml_diff>
--- a/tests/fixtures/smt/synthetic/bom_processed/PLM.xlsx
+++ b/tests/fixtures/smt/synthetic/bom_processed/PLM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -741,7 +741,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Synthetic R0603 component</t>
+          <t>Synthetic C0402 component</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -764,12 +764,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>C0402</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>C0402</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -781,7 +781,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -821,7 +821,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Synthetic C0402 component</t>
+          <t>Synthetic C0603 component</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -844,12 +844,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>C0402</t>
+          <t>C0603</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>C0402</t>
+          <t>C0603</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -861,7 +861,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -901,7 +901,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Synthetic C0603 component</t>
+          <t>Synthetic BGA153 component</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -924,12 +924,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>C0603</t>
+          <t>BGA153</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>C0603</t>
+          <t>BGA153</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -941,7 +941,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Synthetic C0603 component</t>
+          <t>Synthetic QFN48 component</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -964,12 +964,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>C0603</t>
+          <t>QFN48</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>C0603</t>
+          <t>QFN48</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -981,7 +981,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Synthetic BGA153 component</t>
+          <t>Synthetic QFN32 component</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1004,12 +1004,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>BGA153</t>
+          <t>QFN32</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>BGA153</t>
+          <t>QFN32</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1021,7 +1021,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>SH1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Synthetic QFN48 component</t>
+          <t>Synthetic SHIELD_BRACKET component</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1044,12 +1044,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>QFN48</t>
+          <t>SHIELD_BRACKET</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>QFN48</t>
+          <t>SHIELD_BRACKET</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1061,7 +1061,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>JP1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Synthetic QFN32 component</t>
+          <t>Synthetic CONN_2P component</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1084,12 +1084,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>QFN32</t>
+          <t>CONN_2P</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>QFN32</t>
+          <t>CONN_2P</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1101,7 +1101,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SH1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Synthetic SHIELD_BRACKET component</t>
+          <t>Synthetic SOD323 component</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1124,12 +1124,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SHIELD_BRACKET</t>
+          <t>SOD323</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SHIELD_BRACKET</t>
+          <t>SOD323</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1141,7 +1141,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>JP1</t>
+          <t>R99</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Synthetic CONN_2P component</t>
+          <t>Synthetic R0402 component</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1164,135 +1164,15 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>CONN_2P</t>
+          <t>R0402</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>CONN_2P</t>
+          <t>R0402</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
-        <is>
-          <t>优选</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>TP1</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>PN-0019</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Synthetic TESTPOINT component</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>TESTPOINT</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>TESTPOINT</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>优选</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>PN-0020</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Synthetic SOD323 component</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>SOD323</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>SOD323</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>优选</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>R99</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>PN-0021</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Synthetic R0402 component</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>R0402</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>R0402</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
         <is>
           <t>优选</t>
         </is>

</xml_diff>